<commit_message>
Good Working Code Without Error Handling of job Failed Restart were stopped
</commit_message>
<xml_diff>
--- a/Lob_Mapping.xlsx
+++ b/Lob_Mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://exdion-my.sharepoint.com/personal/vijay_m_exdion_com/Documents/Documents/Project_Job_Creation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://exdion-my.sharepoint.com/personal/vijay_m_exdion_com/Documents/Documents/Project_Job_Creation/Carroll/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{9B59C786-FCB3-4E6A-9156-1C3BDC385173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3133015E-5E63-4131-A1D9-3B30BE27B5D7}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{9B59C786-FCB3-4E6A-9156-1C3BDC385173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA1DFBAB-588B-4485-9768-433EDE0A6138}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="14400" windowHeight="7260" xr2:uid="{F1DF3F70-A5FB-4876-B5A3-6DE3CFC4363C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{F1DF3F70-A5FB-4876-B5A3-6DE3CFC4363C}"/>
   </bookViews>
   <sheets>
     <sheet name="Lob_Mapping" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3327" uniqueCount="1372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3330" uniqueCount="1373">
   <si>
     <t>AccDea&amp;Disrem</t>
   </si>
@@ -4152,6 +4152,9 @@
   </si>
   <si>
     <t>LOB_NAME</t>
+  </si>
+  <si>
+    <t>CYBR</t>
   </si>
 </sst>
 </file>
@@ -4216,10 +4219,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4558,7 +4562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2263691B-B4A5-47F0-BD72-5E9ABFD5EDAC}">
-  <dimension ref="A1:C1109"/>
+  <dimension ref="A1:C1110"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.7265625" bestFit="1" customWidth="1"/>
@@ -16765,6 +16769,17 @@
         <v>1366</v>
       </c>
     </row>
+    <row r="1110" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1110" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="B1110" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1110" s="3" t="s">
+        <v>1372</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>